<commit_message>
Corrige la corruption Excel du gabarit RUP : images fantômes orphelines
L'Exemplaire.xlsx source (Aartselaar) avait 10 images incrustées
(icônes décoratives), ancrées sur les colonnes O->AD. delete_cols/
delete_rows d'openpyxl ne met pas à jour la partie XML des dessins
(limitation connue) -- ces images restaient ancrées sur des positions
de colonnes qui n'ont plus le même sens dans le gabarit RUP (colonnes
dynamiques recréées à la volée), rendant le fichier structurellement
incohérent (Excel demandait une réparation à l'ouverture).

- templates/gabarit_rup.xlsx : reconstruit sans aucune image.
- state/8580_avelgem_rup.xlsx : images retirées du fichier déjà produit
  par le run réel (140 rues, 392 lignes) -- données vérifiées
  cellule par cellule, strictement identiques avant/après, seule la
  partie images a changé. Sauvegarde datée du fichier original incluse.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/8580_avelgem_rup.xlsx
+++ b/state/8580_avelgem_rup.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="21480" yWindow="-1905" windowWidth="21840" windowHeight="13020" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RUP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUP" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -196,421 +196,6 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors/>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>100853</colOff>
-      <row>0</row>
-      <rowOff>224118</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>720064</colOff>
-      <row>0</row>
-      <rowOff>643276</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 1"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="16976912" y="224118"/>
-          <a:ext cx="619211" cy="419158"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>20</col>
-      <colOff>40822</colOff>
-      <row>0</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <to>
-      <col>20</col>
-      <colOff>693964</colOff>
-      <row>0</row>
-      <rowOff>556581</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 2"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="22547036" y="95250"/>
-          <a:ext cx="653142" cy="461331"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>21</col>
-      <colOff>748393</colOff>
-      <row>0</row>
-      <rowOff>176893</rowOff>
-    </from>
-    <to>
-      <col>22</col>
-      <colOff>721178</colOff>
-      <row>0</row>
-      <rowOff>585107</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 3"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="23567572" y="176893"/>
-          <a:ext cx="734785" cy="408214"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>25</col>
-      <colOff>680357</colOff>
-      <row>0</row>
-      <rowOff>136071</rowOff>
-    </from>
-    <to>
-      <col>26</col>
-      <colOff>747148</colOff>
-      <row>0</row>
-      <rowOff>540244</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 4"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="26996571" y="136071"/>
-          <a:ext cx="828791" cy="404173"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>27</col>
-      <colOff>81643</colOff>
-      <row>0</row>
-      <rowOff>136071</rowOff>
-    </from>
-    <to>
-      <col>27</col>
-      <colOff>700854</colOff>
-      <row>0</row>
-      <rowOff>518463</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 5"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="27921857" y="136071"/>
-          <a:ext cx="619211" cy="382392"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>100853</colOff>
-      <row>1</row>
-      <rowOff>224118</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>720064</colOff>
-      <row>2</row>
-      <rowOff>71776</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="7" name="Image 1"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="18188828" y="224118"/>
-          <a:ext cx="619211" cy="419158"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>20</col>
-      <colOff>40822</colOff>
-      <row>1</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <to>
-      <col>20</col>
-      <colOff>693964</colOff>
-      <row>1</row>
-      <rowOff>556581</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="8" name="Image 2"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="22538872" y="95250"/>
-          <a:ext cx="653142" cy="461331"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>21</col>
-      <colOff>748393</colOff>
-      <row>1</row>
-      <rowOff>176893</rowOff>
-    </from>
-    <to>
-      <col>22</col>
-      <colOff>721178</colOff>
-      <row>2</row>
-      <rowOff>13607</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 3"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="24008443" y="176893"/>
-          <a:ext cx="734785" cy="408214"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>25</col>
-      <colOff>680357</colOff>
-      <row>1</row>
-      <rowOff>136071</rowOff>
-    </from>
-    <to>
-      <col>26</col>
-      <colOff>747148</colOff>
-      <row>1</row>
-      <rowOff>540244</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 4"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="26988407" y="136071"/>
-          <a:ext cx="828791" cy="404173"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>27</col>
-      <colOff>81643</colOff>
-      <row>1</row>
-      <rowOff>136071</rowOff>
-    </from>
-    <to>
-      <col>27</col>
-      <colOff>700854</colOff>
-      <row>1</row>
-      <rowOff>518463</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 5"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="27913693" y="136071"/>
-          <a:ext cx="619211" cy="382392"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -62843,6 +62428,5 @@
     <mergeCell ref="A325:A335"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Retire la numérotation d'article du texte Bestemming extrait
Vérifié en direct sur les 16 colonnes de l'Exemplaire.xlsx (référence
autoritative) : aucune ne commence par un numéro d'article -- toujours
"Bestemming..."/"Bestemmingsvoorschriften...", jamais "2.1
Bestemming...". rup_pdf_service.py gardait pourtant la numérotation
dans le texte CAPTURÉ (seulement retirée pour la détection du début de
section) -- incohérent avec ce format de référence sur les dossiers
qui numérotent leurs articles (ex. Avelgem). Numérotation retirée du
texte stocké aussi désormais.

state/8580_avelgem_rup.xlsx : les 2 cellules concernées ("zone voor
wonen met beperkte nevenfuncties" et son doublon) corrigées
directement (retrait du préfixe "2.1 ", reste du texte déjà exact et
inchangé). Sauvegarde datée incluse.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/8580_avelgem_rup.xlsx
+++ b/state/8580_avelgem_rup.xlsx
@@ -302,6 +302,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -940,7 +943,7 @@
       </c>
       <c r="O3" s="19" t="inlineStr">
         <is>
-          <t>2.1 Bestemming
+          <t>Bestemming
 De zone is bestemd voor wonen met beperkte nevenfuncties. Binnen deze zone
 zijn wonen en de bijhorende openbare en private groene en verharde ruimten
 de hoofdfuncties. De beperkte nevenfuncties mogen de woonfunctie van de
@@ -1142,7 +1145,7 @@
       </c>
       <c r="AE3" s="19" t="inlineStr">
         <is>
-          <t>2.1 Bestemming
+          <t>Bestemming
 De zone is bestemd voor wonen met beperkte nevenfuncties. Binnen deze
 zone vormen wonen en de bijhorende openbare en private groene en verharde
 ruimten de hoofdfuncties.

</xml_diff>

<commit_message>
Retire la numérotation restante sur les 14 autres colonnes Bestemming
Correctif précédent (7a1c5de) n'avait retiré que le préfixe "2.1 "
trouvé sur 2 colonnes -- en réalité presque toutes les colonnes de
dossiers numérotant leurs articles avaient un préfixe DIFFÉRENT
("5 ", "13 ", "26 ", "9 ", "1 ", "3.1 ", "4.1 ", "5.1 ", "7.1 ", "19 "),
jamais balayé avec l'expression régulière générale déjà utilisée par
le code d'extraction -- signalé par l'utilisateur après vérification
visuelle du fichier. Corrigé sur les 14 colonnes concernées, texte
restant déjà exact et inchangé. Sauvegarde datée incluse.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/8580_avelgem_rup.xlsx
+++ b/state/8580_avelgem_rup.xlsx
@@ -958,7 +958,7 @@
       </c>
       <c r="P3" s="19" t="inlineStr">
         <is>
-          <t>5 Bestemming
+          <t>Bestemming
 De zone is bestemd voor gemeenschapsvoorzieningen.
 Alle werken, handelingen, en wijzigingen die nodig of nuttig zijn voor deze
 bestemmingen zijn toegelaten.</t>
@@ -966,7 +966,7 @@
       </c>
       <c r="Q3" s="19" t="inlineStr">
         <is>
-          <t>13 Bestemming
+          <t>Bestemming
 De zone is bestemd voor service-fl ats.
 Alle werken, handelingen, en wijzigingen die nodig of nuttig zijn voor deze
 bestemming zijn toegelaten.
@@ -977,7 +977,7 @@
       </c>
       <c r="R3" s="19" t="inlineStr">
         <is>
-          <t>26 Bestemming
+          <t>Bestemming
 Het gebied is bestemd voor cultureel-recreatieve functies in open lucht.
 Alle werken, handelingen en wijzigingen die nodig of nuttig zijn voor het
 realiseren van de bestemming, zijn toegelaten.</t>
@@ -985,7 +985,7 @@
       </c>
       <c r="S3" s="19" t="inlineStr">
         <is>
-          <t>26 Bestemming
+          <t>Bestemming
 Het gebied is bestemd voor cultureel-recreatieve functies in open lucht.
 Alle werken, handelingen en wijzigingen die nodig of nuttig zijn voor het
 realiseren van de bestemming, zijn toegelaten.</t>
@@ -993,7 +993,7 @@
       </c>
       <c r="T3" s="19" t="inlineStr">
         <is>
-          <t>9 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor meergezinswoongebouwen (appartementen of
 urban-villa’s) en openbaar groen.
 10 Minimum 40 % van de zone moet ingericht worden als openbaar groengebied.
@@ -1029,7 +1029,7 @@
       </c>
       <c r="U3" s="19" t="inlineStr">
         <is>
-          <t>1 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor de realisatie van een sociaal woonproject met
 aanééngesloten ééngezinswoningen (rijwoningen).
 Indien in de aanpalende zone 2 (zone voor meergezinswoongebouwen en
@@ -1094,7 +1094,7 @@
       </c>
       <c r="AB3" s="19" t="inlineStr">
         <is>
-          <t>3.1 Bestemming
+          <t>Bestemming
 De zone is bestemd voor recreatie.
 Alle werken, handelingen en wijzigingen die nodig of nuttig zijn voor het
 realiseren van deze bestemming, zijn toegelaten.
@@ -1112,7 +1112,7 @@
       </c>
       <c r="AC3" s="19" t="inlineStr">
         <is>
-          <t>3.1 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor openbare wegeninfrastructuur en aanhorigheden.
 3.2 In deze zone zijn alle bovengrondse en ondergrondse werken, handelingen en
 wijzigingen toegelaten voor de aanleg, het functioneren of aanpassing van die
@@ -1128,7 +1128,7 @@
       </c>
       <c r="AD3" s="19" t="inlineStr">
         <is>
-          <t>4.1 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor gemeenschapsvoorzieningen en openbare
 nutsvoorzieningen, met specifi ek het gemeentelijk containerpark (of
 afvalstoffenpark) en de gemeentelijke technische diensten en depot.
@@ -1166,7 +1166,7 @@
       </c>
       <c r="AF3" s="19" t="inlineStr">
         <is>
-          <t>7.1 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor openbare wegeninfrastructuur en aanhorigheden.
 In deze zone zijn alle bovengrondse en ondergrondse werken, handelingen en
 wijzigingen toegelaten voor de aanleg, het functioneren of aanpassing van die
@@ -1179,7 +1179,7 @@
       </c>
       <c r="AG3" s="19" t="inlineStr">
         <is>
-          <t>5.1 Bestemming
+          <t>Bestemming
 De zone is bestemd voor de ontwikkeling en de instandhouding van een
 landschappelijke groenbuffer, eventueel gecombineerd met waterbufferbekkens
 en -infi ltratiezones.
@@ -1192,7 +1192,7 @@
       </c>
       <c r="AH3" s="19" t="inlineStr">
         <is>
-          <t>5.1 Bestemming
+          <t>Bestemming
 De zone is bestemd voor de ontwikkeling en de instandhouding van een
 landschappelijke groenbuffer, eventueel gecombineerd met waterbufferbekkens
 en -infi ltratiezones.
@@ -1205,7 +1205,7 @@
       </c>
       <c r="AI3" s="19" t="inlineStr">
         <is>
-          <t>19 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor gemeenschapsvoorzieningen binnen het oude
 stationsgebouw.
 20 De erfgoedwaarde, het karakter en de architecturale verschijningsvorm van het
@@ -1249,7 +1249,7 @@
       </c>
       <c r="AQ3" s="19" t="inlineStr">
         <is>
-          <t>9 Bestemming
+          <t>Bestemming
 Deze zone is bestemd voor meergezinswoongebouwen (appartementen of
 urban-villa’s) en openbaar groen.
 10 Minimum 40 % van de zone moet ingericht worden als openbaar groengebied.

</xml_diff>